<commit_message>
map-bf-scalability-0.75 results up to 15 tasks, plus tuning study logs
</commit_message>
<xml_diff>
--- a/workspace/framework_paper/map-bf-scalability/map-bf-scalability-0.75/map-bf-scalability-0.75_processed.xlsx
+++ b/workspace/framework_paper/map-bf-scalability/map-bf-scalability-0.75/map-bf-scalability-0.75_processed.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,21 @@
           <t>12</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -477,25 +492,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I2" t="n">
         <v>2</v>
@@ -503,6 +518,15 @@
       <c r="J2" t="n">
         <v>2</v>
       </c>
+      <c r="K2" t="n">
+        <v>2</v>
+      </c>
+      <c r="L2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -511,31 +535,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" t="n">
         <v>14</v>
       </c>
-      <c r="D3" t="n">
-        <v>13</v>
-      </c>
       <c r="E3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F3" t="n">
+        <v>14</v>
+      </c>
+      <c r="G3" t="n">
+        <v>18</v>
+      </c>
+      <c r="H3" t="n">
+        <v>17</v>
+      </c>
+      <c r="I3" t="n">
         <v>16</v>
       </c>
-      <c r="F3" t="n">
-        <v>18</v>
-      </c>
-      <c r="G3" t="n">
-        <v>15</v>
-      </c>
-      <c r="H3" t="n">
-        <v>19</v>
-      </c>
-      <c r="I3" t="n">
-        <v>17</v>
-      </c>
       <c r="J3" t="n">
-        <v>19</v>
+        <v>16</v>
+      </c>
+      <c r="K3" t="n">
+        <v>16</v>
+      </c>
+      <c r="L3" t="n">
+        <v>16</v>
+      </c>
+      <c r="M3" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -545,31 +578,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F4" t="n">
+        <v>16</v>
+      </c>
+      <c r="G4" t="n">
+        <v>22</v>
+      </c>
+      <c r="H4" t="n">
+        <v>18</v>
+      </c>
+      <c r="I4" t="n">
         <v>19</v>
       </c>
-      <c r="G4" t="n">
-        <v>16</v>
-      </c>
-      <c r="H4" t="n">
+      <c r="J4" t="n">
+        <v>21</v>
+      </c>
+      <c r="K4" t="n">
         <v>20</v>
       </c>
-      <c r="I4" t="n">
-        <v>20</v>
-      </c>
-      <c r="J4" t="n">
-        <v>20</v>
+      <c r="L4" t="n">
+        <v>22</v>
+      </c>
+      <c r="M4" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="5">
@@ -579,31 +621,40 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C5" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D5" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E5" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F5" t="n">
         <v>21</v>
       </c>
       <c r="G5" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="H5" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I5" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="J5" t="n">
-        <v>20</v>
+        <v>24</v>
+      </c>
+      <c r="K5" t="n">
+        <v>21</v>
+      </c>
+      <c r="L5" t="n">
+        <v>21</v>
+      </c>
+      <c r="M5" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="6">
@@ -613,31 +664,40 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C6" t="n">
         <v>17</v>
       </c>
       <c r="D6" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E6" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G6" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H6" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I6" t="n">
+        <v>24</v>
+      </c>
+      <c r="J6" t="n">
+        <v>25</v>
+      </c>
+      <c r="K6" t="n">
+        <v>24</v>
+      </c>
+      <c r="L6" t="n">
         <v>23</v>
       </c>
-      <c r="J6" t="n">
-        <v>22</v>
+      <c r="M6" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="7">
@@ -647,31 +707,40 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C7" t="n">
         <v>17</v>
       </c>
       <c r="D7" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E7" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F7" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G7" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I7" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J7" t="n">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="K7" t="n">
+        <v>24</v>
+      </c>
+      <c r="L7" t="n">
+        <v>25</v>
+      </c>
+      <c r="M7" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="8">
@@ -681,31 +750,40 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C8" t="n">
         <v>17</v>
       </c>
       <c r="D8" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E8" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F8" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G8" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H8" t="n">
         <v>25</v>
       </c>
       <c r="I8" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J8" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="K8" t="n">
+        <v>19</v>
+      </c>
+      <c r="L8" t="n">
+        <v>11</v>
+      </c>
+      <c r="M8" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -719,7 +797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -773,6 +851,21 @@
           <t>12</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -781,31 +874,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6.480414886027575e-05</v>
+        <v>3.626599999069395e-05</v>
       </c>
       <c r="C2" t="n">
-        <v>8.326521227982911e-05</v>
+        <v>4.741671427512172e-05</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0001067801245621272</v>
+        <v>7.540283335553492e-05</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0001461039937566966</v>
+        <v>0.0001321748000236767</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0002267320440816028</v>
+        <v>0.000169069666659046</v>
       </c>
       <c r="G2" t="n">
-        <v>0.000344117870554328</v>
+        <v>0.0002102920000197628</v>
       </c>
       <c r="H2" t="n">
-        <v>0.000983052421361208</v>
+        <v>0.0003830970000535672</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0007005000952631235</v>
+        <v>0.0004436250000026121</v>
       </c>
       <c r="J2" t="n">
-        <v>0.0006504370830953121</v>
+        <v>0.001229833499792221</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.000635812499695021</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.001008680333749605</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.0009924580008373596</v>
       </c>
     </row>
     <row r="3">
@@ -815,31 +917,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0005800529933449897</v>
+        <v>0.0005925416666665721</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0002711218715246234</v>
+        <v>0.0002360209166454297</v>
       </c>
       <c r="D3" t="n">
-        <v>0.003861323858682926</v>
+        <v>0.008137467285710695</v>
       </c>
       <c r="E3" t="n">
-        <v>0.003657140492578037</v>
+        <v>0.001840377800006839</v>
       </c>
       <c r="F3" t="n">
-        <v>0.007622168968535132</v>
+        <v>0.0028869018571608</v>
       </c>
       <c r="G3" t="n">
-        <v>0.003508963948115707</v>
+        <v>0.003796745499995622</v>
       </c>
       <c r="H3" t="n">
-        <v>0.008255578798094862</v>
+        <v>0.007679727999997714</v>
       </c>
       <c r="I3" t="n">
-        <v>0.02157315672101343</v>
+        <v>0.01491764568748977</v>
       </c>
       <c r="J3" t="n">
-        <v>0.01214211405941138</v>
+        <v>0.01090138537500707</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.02640961462506652</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.03096703650010113</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.01738334659115605</v>
       </c>
     </row>
     <row r="4">
@@ -849,31 +960,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.02512431430461054</v>
+        <v>0.01890865273331504</v>
       </c>
       <c r="C4" t="n">
-        <v>0.003826282702253333</v>
+        <v>0.006327371846151226</v>
       </c>
       <c r="D4" t="n">
-        <v>0.007633689164112394</v>
+        <v>0.100976605599999</v>
       </c>
       <c r="E4" t="n">
-        <v>0.02773504638496567</v>
+        <v>0.03128871933335328</v>
       </c>
       <c r="F4" t="n">
-        <v>0.15948217750625</v>
+        <v>0.04342568487500387</v>
       </c>
       <c r="G4" t="n">
-        <v>0.04748236725572497</v>
+        <v>0.08366277640909527</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1164220375358127</v>
+        <v>0.077066828833343</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1346854332950898</v>
+        <v>0.1683072499473311</v>
       </c>
       <c r="J4" t="n">
-        <v>0.115126724971924</v>
+        <v>0.0985741426666209</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.2460856354500265</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.9210605096365559</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.3293737192610854</v>
       </c>
     </row>
     <row r="5">
@@ -883,31 +1003,40 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02632078831084073</v>
+        <v>0.01543725775000127</v>
       </c>
       <c r="C5" t="n">
-        <v>0.01786653687903548</v>
+        <v>0.07395857806248074</v>
       </c>
       <c r="D5" t="n">
-        <v>1.213305297854822</v>
+        <v>0.2267668522727397</v>
       </c>
       <c r="E5" t="n">
-        <v>0.5072635525813032</v>
+        <v>0.7522071413043349</v>
       </c>
       <c r="F5" t="n">
-        <v>1.079505914578303</v>
+        <v>4.765122829238105</v>
       </c>
       <c r="G5" t="n">
-        <v>10.8954181074606</v>
+        <v>8.029390501863604</v>
       </c>
       <c r="H5" t="n">
-        <v>6.345412837457843</v>
+        <v>20.40317983527273</v>
       </c>
       <c r="I5" t="n">
-        <v>28.73916021251353</v>
+        <v>31.22757384782608</v>
       </c>
       <c r="J5" t="n">
-        <v>28.55619029167574</v>
+        <v>16.09674671533331</v>
+      </c>
+      <c r="K5" t="n">
+        <v>48.21281959128579</v>
+      </c>
+      <c r="L5" t="n">
+        <v>12.18116302180962</v>
+      </c>
+      <c r="M5" t="n">
+        <v>29.26449824278279</v>
       </c>
     </row>
     <row r="6">
@@ -917,31 +1046,40 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.02859472584289809</v>
+        <v>0.01843572541177122</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0160078578902518</v>
+        <v>0.129810166764688</v>
       </c>
       <c r="D6" t="n">
-        <v>1.297494984231889</v>
+        <v>1.281920262739119</v>
       </c>
       <c r="E6" t="n">
-        <v>1.42670874184696</v>
+        <v>0.7394477444347806</v>
       </c>
       <c r="F6" t="n">
-        <v>1.327091056737117</v>
+        <v>5.205924701043465</v>
       </c>
       <c r="G6" t="n">
-        <v>17.85582339488679</v>
+        <v>9.299666642250008</v>
       </c>
       <c r="H6" t="n">
-        <v>13.34420926197033</v>
+        <v>34.89968002369567</v>
       </c>
       <c r="I6" t="n">
-        <v>31.81298018841114</v>
+        <v>30.30948313891664</v>
       </c>
       <c r="J6" t="n">
-        <v>51.42500708514655</v>
+        <v>15.20643943663998</v>
+      </c>
+      <c r="K6" t="n">
+        <v>56.36804600862496</v>
+      </c>
+      <c r="L6" t="n">
+        <v>18.38217407795653</v>
+      </c>
+      <c r="M6" t="n">
+        <v>47.13157558845857</v>
       </c>
     </row>
     <row r="7">
@@ -951,31 +1089,40 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.026301715328979</v>
+        <v>0.02235780876471568</v>
       </c>
       <c r="C7" t="n">
-        <v>0.02061009796007591</v>
+        <v>0.1458173823529358</v>
       </c>
       <c r="D7" t="n">
-        <v>1.512699148728557</v>
+        <v>1.568116256958324</v>
       </c>
       <c r="E7" t="n">
-        <v>1.47097353747813</v>
+        <v>0.3944933299583179</v>
       </c>
       <c r="F7" t="n">
-        <v>1.414959251944145</v>
+        <v>6.872146368083331</v>
       </c>
       <c r="G7" t="n">
-        <v>12.84765641076402</v>
+        <v>7.009271557416649</v>
       </c>
       <c r="H7" t="n">
-        <v>8.142775484826416</v>
+        <v>21.47181274469565</v>
       </c>
       <c r="I7" t="n">
-        <v>34.80533939487625</v>
+        <v>30.37568633152002</v>
       </c>
       <c r="J7" t="n">
-        <v>58.57394946984608</v>
+        <v>24.15656296827998</v>
+      </c>
+      <c r="K7" t="n">
+        <v>57.52374742183336</v>
+      </c>
+      <c r="L7" t="n">
+        <v>29.68514622004011</v>
+      </c>
+      <c r="M7" t="n">
+        <v>43.55049703824974</v>
       </c>
     </row>
     <row r="8">
@@ -985,31 +1132,40 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.001645017279467235</v>
+        <v>0.001141102999982275</v>
       </c>
       <c r="C8" t="n">
-        <v>0.009387249962481506</v>
+        <v>0.003903406941162757</v>
       </c>
       <c r="D8" t="n">
-        <v>0.06007118051916006</v>
+        <v>0.0301499895833454</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9868328770601444</v>
+        <v>0.470464069374998</v>
       </c>
       <c r="F8" t="n">
-        <v>0.4318673560311171</v>
+        <v>0.3283346567200078</v>
       </c>
       <c r="G8" t="n">
-        <v>0.3326149384146961</v>
+        <v>0.3626476766400037</v>
       </c>
       <c r="H8" t="n">
-        <v>1.729736743345857</v>
+        <v>1.774079328440002</v>
       </c>
       <c r="I8" t="n">
-        <v>10.35234041859234</v>
+        <v>11.43179274996002</v>
       </c>
       <c r="J8" t="n">
-        <v>130.8133811736285</v>
+        <v>172.48849614332</v>
+      </c>
+      <c r="K8" t="n">
+        <v>515.5375197917896</v>
+      </c>
+      <c r="L8" t="n">
+        <v>620.443552007727</v>
+      </c>
+      <c r="M8" t="n">
+        <v>703.8849593166008</v>
       </c>
     </row>
   </sheetData>
@@ -1023,7 +1179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1077,6 +1233,21 @@
           <t>12</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1111,6 +1282,15 @@
       <c r="J2" t="n">
         <v>25</v>
       </c>
+      <c r="K2" t="n">
+        <v>25</v>
+      </c>
+      <c r="L2" t="n">
+        <v>25</v>
+      </c>
+      <c r="M2" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1145,6 +1325,15 @@
       <c r="J3" t="n">
         <v>25</v>
       </c>
+      <c r="K3" t="n">
+        <v>25</v>
+      </c>
+      <c r="L3" t="n">
+        <v>25</v>
+      </c>
+      <c r="M3" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1179,6 +1368,15 @@
       <c r="J4" t="n">
         <v>25</v>
       </c>
+      <c r="K4" t="n">
+        <v>25</v>
+      </c>
+      <c r="L4" t="n">
+        <v>25</v>
+      </c>
+      <c r="M4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1213,6 +1411,15 @@
       <c r="J5" t="n">
         <v>25</v>
       </c>
+      <c r="K5" t="n">
+        <v>25</v>
+      </c>
+      <c r="L5" t="n">
+        <v>25</v>
+      </c>
+      <c r="M5" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1245,7 +1452,16 @@
         <v>25</v>
       </c>
       <c r="J6" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="K6" t="n">
+        <v>25</v>
+      </c>
+      <c r="L6" t="n">
+        <v>25</v>
+      </c>
+      <c r="M6" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="7">
@@ -1279,7 +1495,16 @@
         <v>25</v>
       </c>
       <c r="J7" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="K7" t="n">
+        <v>25</v>
+      </c>
+      <c r="L7" t="n">
+        <v>25</v>
+      </c>
+      <c r="M7" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="8">
@@ -1310,10 +1535,19 @@
         <v>25</v>
       </c>
       <c r="I8" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J8" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="K8" t="n">
+        <v>19</v>
+      </c>
+      <c r="L8" t="n">
+        <v>11</v>
+      </c>
+      <c r="M8" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>